<commit_message>
Update affiliations in validation data and related files
</commit_message>
<xml_diff>
--- a/downloads/AeroSafe_Questionnaire_Answers_Full.xlsx
+++ b/downloads/AeroSafe_Questionnaire_Answers_Full.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alberto.petrucci\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albertopetrucci/Documents/github/aerosafe/downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF9FDCA-466C-2A49-A98E-D7063255C88B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="495" windowWidth="38400" windowHeight="21105" activeTab="1"/>
+    <workbookView xWindow="38400" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AeroSafe Questionnaire Answers" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary Table'!$A$1:$M$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -98,9 +99,6 @@
     <t>0–2 years (Junior / Early career)</t>
   </si>
   <si>
-    <t>Thales Alenia Space</t>
-  </si>
-  <si>
     <t>It is not clear which level is concerned for these reviews : system, subsystem, AI/ML constituent?</t>
   </si>
   <si>
@@ -1256,11 +1254,14 @@
   <si>
     <t>To what extent do you agree that pre-deployment tests for unintended behaviour are sufficient for critical systems (B and A)?</t>
   </si>
+  <si>
+    <t>Space Company</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
@@ -1413,7 +1414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1436,12 +1437,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1458,9 +1453,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1471,12 +1463,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1497,54 +1483,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1560,11 +1498,87 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="86">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2794,16 +2808,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -2855,7 +2859,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="Risposte del modulo 1-style" pivot="0" count="5">
+    <tableStyle name="Risposte del modulo 1-style" pivot="0" count="5" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" size="0" dxfId="85"/>
       <tableStyleElement type="headerRow" dxfId="84"/>
       <tableStyleElement type="totalRow" dxfId="83"/>
@@ -2875,7 +2879,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Risposte del modulo 1"/>
@@ -2915,46 +2919,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A2:AL8" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78" totalsRowDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A2:AL8" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79" totalsRowDxfId="78">
   <tableColumns count="38">
-    <tableColumn id="1" name="Informazioni cronologiche" dataDxfId="76" totalsRowDxfId="75"/>
-    <tableColumn id="30" name="Expert ID" dataDxfId="74" totalsRowDxfId="73"/>
-    <tableColumn id="2" name="Please indicate your professional background (select one or specify)" dataDxfId="72" totalsRowDxfId="71"/>
-    <tableColumn id="3" name="Years of experience in your field" dataDxfId="70" totalsRowDxfId="69"/>
-    <tableColumn id="4" name="Experience with ECSS standards" dataDxfId="68" totalsRowDxfId="67"/>
-    <tableColumn id="5" name="Experience with AI/ML systems" dataDxfId="66" totalsRowDxfId="65"/>
-    <tableColumn id="6" name="Please indicate the name of the organization or company you are currently employed by" dataDxfId="64" totalsRowDxfId="63"/>
-    <tableColumn id="7" name="If you selected “Other”, please specify the organization or company you work for: " dataDxfId="62" totalsRowDxfId="61"/>
-    <tableColumn id="8" name="To what extent do you agree that the following three phases (TRR, CDR, VVR) are sufficient for software qualification and follow the ECSS standards?" dataDxfId="60" totalsRowDxfId="59"/>
-    <tableColumn id="9" name="Are there any important missing elements in the proposed review phases? If so, please specify." dataDxfId="58" totalsRowDxfId="57"/>
-    <tableColumn id="10" name="To what extent do you agree that the proposed configuration management phases (version control, change management, baseline management, traceability) are sufficient and follow the ECSS standard?" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="11" name="Are there any important missing elements in the proposed review phases? If so, please specify. 2" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="12" name="To what extent do you agree that the dataset quality verification process is sufficient for AI applications?" dataDxfId="52" totalsRowDxfId="51"/>
-    <tableColumn id="13" name="Do you have additional considerations for bias mitigation, security, and privacy in satellite applications? If so, please specify." dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="14" name="To what extent do you agree that the proposed methodologies (e.g., data leakage, data mismatch, drift analysis) are necessary to ensure model quality during the learning phase, considering criticality levels?" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="15" name="To what extent do you agree that model performance validation is sufficient to ensure model quality during the learning phase, considering criticality levels?" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="16" name="To what extent do you agree that model explainability and bias/fairness audits help to qualify a model with the highest criticality level?" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="17" name="Are there any important missing elements in the proposed review phases? If so, please specify. 3" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="18" name="To what extent do you agree that the proposed verification methodologies (e.g., formal methods, robustness testing) are necessary to ensure model quality during the verification phase, considering criticality levels?" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="19" name="To what extent do you agree that generating test cases from the design domain and that simulation-based testing are necessary to ensure model quality during the verification phase, considering criticality levels?" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="20" name="To what extent do you agree that adversarial robustness testing and stress testing should be mandatory for A-critical systems?" dataDxfId="36" totalsRowDxfId="35"/>
-    <tableColumn id="21" name="Are there any important missing elements in the proposed review phases? If so, please specify. 4" dataDxfId="34" totalsRowDxfId="33"/>
-    <tableColumn id="22" name="To what extent do you agree that embeddability is a critical factor for model selection and design, especially for deployment on embedded hardware?" dataDxfId="32" totalsRowDxfId="31"/>
-    <tableColumn id="23" name="To what extent do you agree that using integrated development environments (from GPU-based development/testing to real-target deployment) impacts qualification?" dataDxfId="30" totalsRowDxfId="29"/>
-    <tableColumn id="24" name="To what extent do you agree that pre and post deployment validation and monitoring is important to qualify critical models?" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="25" name="To what extent do you agree that model obsolescence is a risk, and that defining an update plan is important?" dataDxfId="26" totalsRowDxfId="25"/>
-    <tableColumn id="26" name="For critical applications, to what extent do you agree that feedback loop in model design improves model continuous improvement?_x000a__x000a_Feedback Loops: Establish mechanisms to collect feedback from users or systems to continuously improve the model in order to " dataDxfId="24" totalsRowDxfId="23"/>
-    <tableColumn id="27" name="For critical applications, to what extent do you agree that redundancy improves robustness? What do you consider the right trade-off between robustness and resource usage?" dataDxfId="22" totalsRowDxfId="21"/>
-    <tableColumn id="28" name="To what extent do you agree that real-time model monitoring (e.g., for model drift or failures) should be mandatory for A-critical systems?" dataDxfId="20" totalsRowDxfId="19"/>
-    <tableColumn id="29" name="Are there any important missing elements in the proposed review phases? If so, please specify. 5" dataDxfId="18" totalsRowDxfId="17"/>
-    <tableColumn id="32" name="To what extent do you agree that the proposed integration and traceability questions are sufficient to ensure consistency across lifecycle phases?" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="33" name="Are there any important missing elements in the proposed review phases? If so, please specify. 7" dataDxfId="14" totalsRowDxfId="13"/>
-    <tableColumn id="34" name="To what extent do you agree that external requirement verification is sufficient for critical systems (B and A)?" dataDxfId="12" totalsRowDxfId="11"/>
-    <tableColumn id="35" name="To what extent do you agree that external validation of training data and models is sufficient for critical systems (B and A)?" dataDxfId="10" totalsRowDxfId="9"/>
-    <tableColumn id="36" name="To what extent do you agree that pre-deployment tests for unintended behaviour are sufficient for critical systems (B and A)?" dataDxfId="8" totalsRowDxfId="7"/>
-    <tableColumn id="37" name="To what extent do you agree that continuous monitoring and recertification should be mandatory for post-deployment?" dataDxfId="6" totalsRowDxfId="5"/>
-    <tableColumn id="38" name="To what extent do you agree that regulatory conformance checks should be mandatory for A-critical systems?" dataDxfId="4" totalsRowDxfId="3"/>
-    <tableColumn id="39" name="Are there any important missing elements in the proposed review phases? If so, please specify. 8" dataDxfId="2" totalsRowDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Informazioni cronologiche" dataDxfId="77" totalsRowDxfId="76"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Expert ID" dataDxfId="75" totalsRowDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Please indicate your professional background (select one or specify)" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Years of experience in your field" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Experience with ECSS standards" dataDxfId="69" totalsRowDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Experience with AI/ML systems" dataDxfId="67" totalsRowDxfId="66"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Please indicate the name of the organization or company you are currently employed by" dataDxfId="65" totalsRowDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="If you selected “Other”, please specify the organization or company you work for: " dataDxfId="63" totalsRowDxfId="62"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="To what extent do you agree that the following three phases (TRR, CDR, VVR) are sufficient for software qualification and follow the ECSS standards?" dataDxfId="61" totalsRowDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify." dataDxfId="59" totalsRowDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="To what extent do you agree that the proposed configuration management phases (version control, change management, baseline management, traceability) are sufficient and follow the ECSS standard?" dataDxfId="57" totalsRowDxfId="56"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 2" dataDxfId="55" totalsRowDxfId="54"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="To what extent do you agree that the dataset quality verification process is sufficient for AI applications?" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Do you have additional considerations for bias mitigation, security, and privacy in satellite applications? If so, please specify." dataDxfId="51" totalsRowDxfId="50"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="To what extent do you agree that the proposed methodologies (e.g., data leakage, data mismatch, drift analysis) are necessary to ensure model quality during the learning phase, considering criticality levels?" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="To what extent do you agree that model performance validation is sufficient to ensure model quality during the learning phase, considering criticality levels?" dataDxfId="47" totalsRowDxfId="46"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="To what extent do you agree that model explainability and bias/fairness audits help to qualify a model with the highest criticality level?" dataDxfId="45" totalsRowDxfId="44"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 3" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="To what extent do you agree that the proposed verification methodologies (e.g., formal methods, robustness testing) are necessary to ensure model quality during the verification phase, considering criticality levels?" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="To what extent do you agree that generating test cases from the design domain and that simulation-based testing are necessary to ensure model quality during the verification phase, considering criticality levels?" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="To what extent do you agree that adversarial robustness testing and stress testing should be mandatory for A-critical systems?" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 4" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="To what extent do you agree that embeddability is a critical factor for model selection and design, especially for deployment on embedded hardware?" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="To what extent do you agree that using integrated development environments (from GPU-based development/testing to real-target deployment) impacts qualification?" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="To what extent do you agree that pre and post deployment validation and monitoring is important to qualify critical models?" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="To what extent do you agree that model obsolescence is a risk, and that defining an update plan is important?" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="For critical applications, to what extent do you agree that feedback loop in model design improves model continuous improvement?_x000a__x000a_Feedback Loops: Establish mechanisms to collect feedback from users or systems to continuously improve the model in order to " dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="For critical applications, to what extent do you agree that redundancy improves robustness? What do you consider the right trade-off between robustness and resource usage?" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="To what extent do you agree that real-time model monitoring (e.g., for model drift or failures) should be mandatory for A-critical systems?" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 5" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="To what extent do you agree that the proposed integration and traceability questions are sufficient to ensure consistency across lifecycle phases?" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 7" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="To what extent do you agree that external requirement verification is sufficient for critical systems (B and A)?" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="To what extent do you agree that external validation of training data and models is sufficient for critical systems (B and A)?" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="To what extent do you agree that pre-deployment tests for unintended behaviour are sufficient for critical systems (B and A)?" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="To what extent do you agree that continuous monitoring and recertification should be mandatory for post-deployment?" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="To what extent do you agree that regulatory conformance checks should be mandatory for A-critical systems?" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Are there any important missing elements in the proposed review phases? If so, please specify. 8" dataDxfId="3" totalsRowDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3157,78 +3161,78 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AL9"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="2" width="24.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="37.7109375" style="6" customWidth="1"/>
-    <col min="4" max="4" width="28.28515625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="28.7109375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="28.140625" style="6" customWidth="1"/>
-    <col min="7" max="37" width="37.7109375" style="6" customWidth="1"/>
-    <col min="38" max="38" width="187.7109375" style="6" customWidth="1"/>
-    <col min="39" max="44" width="18.85546875" style="6" customWidth="1"/>
-    <col min="45" max="16384" width="12.7109375" style="6"/>
+    <col min="1" max="2" width="24.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="28.33203125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="28.1640625" style="6" customWidth="1"/>
+    <col min="7" max="37" width="37.6640625" style="6" customWidth="1"/>
+    <col min="38" max="38" width="187.6640625" style="6" customWidth="1"/>
+    <col min="39" max="44" width="18.83203125" style="6" customWidth="1"/>
+    <col min="45" max="16384" width="12.6640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="I1" s="8" t="s">
+    <row r="1" spans="1:38" s="1" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="I1" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="29"/>
+      <c r="K1" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="30"/>
+      <c r="M1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="9"/>
-      <c r="M1" s="8" t="s">
+      <c r="N1" s="29"/>
+      <c r="O1" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="N1" s="8"/>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="8" t="s">
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF1" s="29"/>
+      <c r="AG1" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9"/>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
-      <c r="AE1" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH1" s="9"/>
-      <c r="AI1" s="9"/>
-      <c r="AJ1" s="9"/>
-      <c r="AK1" s="9"/>
-      <c r="AL1" s="9"/>
+      <c r="AH1" s="30"/>
+      <c r="AI1" s="30"/>
+      <c r="AJ1" s="30"/>
+      <c r="AK1" s="30"/>
+      <c r="AL1" s="30"/>
     </row>
-    <row r="2" spans="1:38" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:38" ht="98" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>1</v>
@@ -3246,7 +3250,7 @@
         <v>5</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>6</v>
@@ -3255,96 +3259,96 @@
         <v>7</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="M2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="W2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="X2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" s="2" t="s">
+      <c r="AA2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AB2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AA2" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AH2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AI2" s="2" t="s">
+      <c r="AK2" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AJ2" s="2" t="s">
+      <c r="AL2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AK2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>74</v>
-      </c>
     </row>
-    <row r="3" spans="1:38" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:38" ht="28" x14ac:dyDescent="0.15">
       <c r="A3" s="3">
         <v>45967.376392997685</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>9</v>
@@ -3445,12 +3449,12 @@
       </c>
       <c r="AL3" s="4"/>
     </row>
-    <row r="4" spans="1:38" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:38" ht="84" x14ac:dyDescent="0.15">
       <c r="A4" s="3">
         <v>45967.741526400467</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>16</v>
@@ -3465,106 +3469,106 @@
         <v>18</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4">
         <v>5</v>
       </c>
       <c r="J4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4">
+        <v>5</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="4">
-        <v>5</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="M4" s="4">
+        <v>5</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="4">
-        <v>5</v>
-      </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="4">
+        <v>5</v>
+      </c>
+      <c r="P4" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>5</v>
+      </c>
+      <c r="R4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="O4" s="4">
-        <v>5</v>
-      </c>
-      <c r="P4" s="4">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="4">
-        <v>5</v>
-      </c>
-      <c r="R4" s="5" t="s">
+      <c r="S4" s="4">
+        <v>5</v>
+      </c>
+      <c r="T4" s="4">
+        <v>5</v>
+      </c>
+      <c r="U4" s="4">
+        <v>5</v>
+      </c>
+      <c r="V4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="4">
-        <v>5</v>
-      </c>
-      <c r="T4" s="4">
-        <v>5</v>
-      </c>
-      <c r="U4" s="4">
-        <v>5</v>
-      </c>
-      <c r="V4" s="5" t="s">
+      <c r="W4" s="4">
+        <v>5</v>
+      </c>
+      <c r="X4" s="4">
+        <v>5</v>
+      </c>
+      <c r="Y4" s="4">
+        <v>5</v>
+      </c>
+      <c r="Z4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AA4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AB4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AC4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AD4" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="W4" s="4">
-        <v>5</v>
-      </c>
-      <c r="X4" s="4">
-        <v>5</v>
-      </c>
-      <c r="Y4" s="4">
-        <v>5</v>
-      </c>
-      <c r="Z4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AA4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AB4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AC4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AD4" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="AE4" s="4">
         <v>3</v>
       </c>
       <c r="AF4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AG4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AH4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AI4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AJ4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AK4" s="4">
+        <v>5</v>
+      </c>
+      <c r="AL4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AG4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AH4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AI4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AJ4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AK4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AL4" s="5" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="5" spans="1:38" ht="409.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:38" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A5" s="3">
         <v>45971.561985208333</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>16</v>
@@ -3579,105 +3583,105 @@
         <v>18</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="I5" s="4">
         <v>5</v>
       </c>
       <c r="J5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="4">
+        <v>5</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="4">
-        <v>5</v>
-      </c>
-      <c r="L5" s="5" t="s">
+      <c r="M5" s="4">
+        <v>4</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M5" s="4">
-        <v>4</v>
-      </c>
-      <c r="N5" s="5" t="s">
+      <c r="O5" s="4">
+        <v>4</v>
+      </c>
+      <c r="P5" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>4</v>
+      </c>
+      <c r="R5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="O5" s="4">
-        <v>4</v>
-      </c>
-      <c r="P5" s="4">
-        <v>4</v>
-      </c>
-      <c r="Q5" s="4">
-        <v>4</v>
-      </c>
-      <c r="R5" s="5" t="s">
+      <c r="S5" s="4">
+        <v>5</v>
+      </c>
+      <c r="T5" s="4">
+        <v>5</v>
+      </c>
+      <c r="U5" s="4">
+        <v>5</v>
+      </c>
+      <c r="V5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="S5" s="4">
-        <v>5</v>
-      </c>
-      <c r="T5" s="4">
-        <v>5</v>
-      </c>
-      <c r="U5" s="4">
-        <v>5</v>
-      </c>
-      <c r="V5" s="5" t="s">
+      <c r="W5" s="4">
+        <v>5</v>
+      </c>
+      <c r="X5" s="4">
+        <v>4</v>
+      </c>
+      <c r="Y5" s="4">
+        <v>5</v>
+      </c>
+      <c r="Z5" s="4">
+        <v>4</v>
+      </c>
+      <c r="AA5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AB5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AC5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AD5" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="W5" s="4">
-        <v>5</v>
-      </c>
-      <c r="X5" s="4">
-        <v>4</v>
-      </c>
-      <c r="Y5" s="4">
-        <v>5</v>
-      </c>
-      <c r="Z5" s="4">
-        <v>4</v>
-      </c>
-      <c r="AA5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AB5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AC5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AD5" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="AE5" s="4">
         <v>3</v>
       </c>
       <c r="AF5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AG5" s="4">
+        <v>4</v>
+      </c>
+      <c r="AH5" s="4">
+        <v>4</v>
+      </c>
+      <c r="AI5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AJ5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AK5" s="4">
+        <v>5</v>
+      </c>
+      <c r="AL5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AG5" s="4">
-        <v>4</v>
-      </c>
-      <c r="AH5" s="4">
-        <v>4</v>
-      </c>
-      <c r="AI5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AJ5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AK5" s="4">
-        <v>5</v>
-      </c>
-      <c r="AL5" s="5" t="s">
-        <v>35</v>
-      </c>
     </row>
-    <row r="6" spans="1:38" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:38" ht="126" x14ac:dyDescent="0.15">
       <c r="A6" s="3">
         <v>45978.406877465277</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>16</v>
@@ -3692,13 +3696,13 @@
         <v>18</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>
@@ -3716,7 +3720,7 @@
         <v>3</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="S6" s="4">
         <v>5</v>
@@ -3749,14 +3753,14 @@
         <v>5</v>
       </c>
       <c r="AD6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE6" s="4">
+        <v>5</v>
+      </c>
+      <c r="AF6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AE6" s="4">
-        <v>5</v>
-      </c>
-      <c r="AF6" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="AG6" s="4">
         <v>5</v>
       </c>
@@ -3773,12 +3777,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:38" ht="14" x14ac:dyDescent="0.15">
       <c r="A7" s="3">
         <v>45980.494660706019</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>16</v>
@@ -3793,13 +3797,13 @@
         <v>18</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="I7" s="4">
         <v>4</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K7" s="4">
         <v>5</v>
@@ -3865,15 +3869,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:38" ht="14" x14ac:dyDescent="0.15">
       <c r="A8" s="3">
         <v>45991.355830671295</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>18</v>
@@ -3885,7 +3889,7 @@
         <v>10</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="I8" s="4">
         <v>3</v>
@@ -3954,90 +3958,90 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:38" s="7" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="C9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="K9" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="M9" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="O9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="P9" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="Q9" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="Q9" s="7" t="s">
+      <c r="S9" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="S9" s="7" t="s">
+      <c r="T9" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="T9" s="7" t="s">
+      <c r="U9" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="U9" s="7" t="s">
+      <c r="W9" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="W9" s="7" t="s">
+      <c r="X9" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="X9" s="7" t="s">
+      <c r="Y9" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="Y9" s="7" t="s">
+      <c r="Z9" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="Z9" s="7" t="s">
+      <c r="AA9" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="AA9" s="7" t="s">
+      <c r="AB9" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="AB9" s="7" t="s">
+      <c r="AC9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="AC9" s="7" t="s">
+      <c r="AE9" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="AE9" s="7" t="s">
+      <c r="AG9" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="AG9" s="7" t="s">
+      <c r="AH9" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="AH9" s="7" t="s">
+      <c r="AI9" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="AI9" s="7" t="s">
+      <c r="AJ9" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="AJ9" s="7" t="s">
+      <c r="AK9" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="AK9" s="7" t="s">
-        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -4052,7 +4056,7 @@
     <mergeCell ref="M1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:AL8">
-    <cfRule type="cellIs" dxfId="80" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="between">
       <formula>2</formula>
       <formula>3</formula>
     </cfRule>
@@ -4065,1096 +4069,1102 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M29"/>
-  <sheetFormatPr defaultColWidth="49.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="49.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="46" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" style="47" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="29.85546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28" style="48" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.140625" style="48" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" style="49" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.7109375" style="48" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7" style="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="49.85546875" style="13"/>
+    <col min="1" max="1" width="22.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.33203125" style="26" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="29.83203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.1640625" style="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.1640625" style="28" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.6640625" style="27" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7" style="11" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="49.83203125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+      <c r="A1" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="I1" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="J1" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="K1" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="L1" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="M1" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="M1" s="14" t="s">
+    </row>
+    <row r="2" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+      <c r="A2" s="31" t="s">
         <v>127</v>
       </c>
+      <c r="B2" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="16"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="B2" s="17" t="s">
+    <row r="3" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+      <c r="A3" s="32"/>
+      <c r="B3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="21"/>
-      <c r="B3" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="19">
+      <c r="J3" s="16">
         <f>AVERAGE(VLOOKUP(D3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I3,[1]Values!$A$2:$B$4,2,0))</f>
         <v>7.5</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="19">
+      <c r="K3" s="17"/>
+      <c r="L3" s="16">
         <f>STDEV(VLOOKUP(D3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H3,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I3,[1]Values!$A$2:$B$4,2,0))</f>
         <v>6.6858058601787116</v>
       </c>
-      <c r="M3" s="19"/>
+      <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="21"/>
-      <c r="B4" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="18" t="s">
+    <row r="4" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+      <c r="A4" s="32"/>
+      <c r="B4" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="I4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="19">
+      <c r="J4" s="16">
         <f>AVERAGE(VLOOKUP(D4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I4,[1]Values!$A$2:$B$4,2,0))</f>
         <v>7</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="19">
+      <c r="K4" s="17"/>
+      <c r="L4" s="16">
         <f>STDEV(VLOOKUP(D4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H4,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I4,[1]Values!$A$2:$B$4,2,0))</f>
         <v>7.0992957397195395</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="16"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="21"/>
-      <c r="B5" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="17" t="s">
+    <row r="5" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+      <c r="A5" s="32"/>
+      <c r="B5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="I5" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="16">
         <f>AVERAGE(VLOOKUP(D5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I5,[1]Values!$A$2:$B$4,2,0))</f>
         <v>2</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="19">
+      <c r="K5" s="17"/>
+      <c r="L5" s="16">
         <f>STDEV(VLOOKUP(D5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(E5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(F5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(G5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(H5,[1]Values!$A$2:$B$4,2,0),VLOOKUP(I5,[1]Values!$A$2:$B$4,2,0))</f>
         <v>1.5491933384829668</v>
       </c>
-      <c r="M5" s="19"/>
+      <c r="M5" s="16"/>
     </row>
-    <row r="6" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="21"/>
-      <c r="B6" s="17" t="s">
+    <row r="6" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A6" s="32"/>
+      <c r="B6" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="G6" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="H6" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="I6" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="J6" s="16"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+    </row>
+    <row r="7" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A7" s="33"/>
+      <c r="B7" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="19"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
+      <c r="C7" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
     </row>
-    <row r="7" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
-      <c r="B7" s="17" t="s">
+    <row r="8" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A8" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-    </row>
-    <row r="8" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="24">
-        <v>4</v>
-      </c>
-      <c r="E8" s="24">
-        <v>5</v>
-      </c>
-      <c r="F8" s="24">
-        <v>5</v>
-      </c>
-      <c r="G8" s="24">
+      <c r="D8" s="19">
+        <v>4</v>
+      </c>
+      <c r="E8" s="19">
+        <v>5</v>
+      </c>
+      <c r="F8" s="19">
+        <v>5</v>
+      </c>
+      <c r="G8" s="19">
         <v>3</v>
       </c>
-      <c r="H8" s="24">
-        <v>4</v>
-      </c>
-      <c r="I8" s="24">
+      <c r="H8" s="19">
+        <v>4</v>
+      </c>
+      <c r="I8" s="19">
         <v>3</v>
       </c>
-      <c r="J8" s="26">
+      <c r="J8" s="21">
         <f t="shared" ref="J8:J29" si="0">AVERAGE(D8:I8)</f>
         <v>4</v>
       </c>
-      <c r="K8" s="27">
+      <c r="K8" s="49">
         <f>AVERAGE(J8:J9)</f>
         <v>4.25</v>
       </c>
-      <c r="L8" s="26">
+      <c r="L8" s="21">
         <f>STDEV(D8:I8)</f>
         <v>0.89442719099991586</v>
       </c>
-      <c r="M8" s="26">
+      <c r="M8" s="21">
         <f>QUARTILE(E8:J8,3)-QUARTILE(E8:J8,1)</f>
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A9" s="28" t="s">
+    <row r="9" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A9" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="D9" s="17">
-        <v>4</v>
-      </c>
-      <c r="E9" s="17">
-        <v>5</v>
-      </c>
-      <c r="F9" s="17">
-        <v>5</v>
-      </c>
-      <c r="G9" s="17">
-        <v>5</v>
-      </c>
-      <c r="H9" s="17">
-        <v>5</v>
-      </c>
-      <c r="I9" s="17">
+      <c r="D9" s="14">
+        <v>4</v>
+      </c>
+      <c r="E9" s="14">
+        <v>5</v>
+      </c>
+      <c r="F9" s="14">
+        <v>5</v>
+      </c>
+      <c r="G9" s="14">
+        <v>5</v>
+      </c>
+      <c r="H9" s="14">
+        <v>5</v>
+      </c>
+      <c r="I9" s="14">
         <v>3</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="16">
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
-      <c r="K9" s="27"/>
-      <c r="L9" s="19">
+      <c r="K9" s="49"/>
+      <c r="L9" s="16">
         <f>STDEV(D9:I9)</f>
         <v>0.83666002653407556</v>
       </c>
-      <c r="M9" s="19">
+      <c r="M9" s="16">
         <f>QUARTILE(E9:J9,3)-QUARTILE(E9:J9,1)</f>
         <v>0.375</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A10" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="D10" s="24">
-        <v>4</v>
-      </c>
-      <c r="E10" s="24">
-        <v>5</v>
-      </c>
-      <c r="F10" s="24">
-        <v>4</v>
-      </c>
-      <c r="G10" s="24">
-        <v>4</v>
-      </c>
-      <c r="H10" s="24">
-        <v>5</v>
-      </c>
-      <c r="I10" s="24">
-        <v>4</v>
-      </c>
-      <c r="J10" s="26">
+      <c r="D10" s="19">
+        <v>4</v>
+      </c>
+      <c r="E10" s="19">
+        <v>5</v>
+      </c>
+      <c r="F10" s="19">
+        <v>4</v>
+      </c>
+      <c r="G10" s="19">
+        <v>4</v>
+      </c>
+      <c r="H10" s="19">
+        <v>5</v>
+      </c>
+      <c r="I10" s="19">
+        <v>4</v>
+      </c>
+      <c r="J10" s="21">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K10" s="29">
+      <c r="K10" s="22">
         <f>AVERAGE(D10:I10)</f>
         <v>4.333333333333333</v>
       </c>
-      <c r="L10" s="26">
+      <c r="L10" s="21">
         <f>STDEV(D10:I10)</f>
         <v>0.51639777949432131</v>
       </c>
-      <c r="M10" s="26">
+      <c r="M10" s="21">
         <f>QUARTILE(E10:J10,3)-QUARTILE(E10:J10,1)</f>
         <v>0.83333333333333304</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A11" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="B11" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="D11" s="17">
-        <v>5</v>
-      </c>
-      <c r="E11" s="17">
-        <v>5</v>
-      </c>
-      <c r="F11" s="17">
-        <v>4</v>
-      </c>
-      <c r="G11" s="17">
-        <v>5</v>
-      </c>
-      <c r="H11" s="17">
-        <v>5</v>
-      </c>
-      <c r="I11" s="17">
-        <v>4</v>
-      </c>
-      <c r="J11" s="19">
+      <c r="D11" s="14">
+        <v>5</v>
+      </c>
+      <c r="E11" s="14">
+        <v>5</v>
+      </c>
+      <c r="F11" s="14">
+        <v>4</v>
+      </c>
+      <c r="G11" s="14">
+        <v>5</v>
+      </c>
+      <c r="H11" s="14">
+        <v>5</v>
+      </c>
+      <c r="I11" s="14">
+        <v>4</v>
+      </c>
+      <c r="J11" s="16">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="34">
         <f>AVERAGE(J11:J13)</f>
         <v>4.2222222222222223</v>
       </c>
-      <c r="L11" s="31">
+      <c r="L11" s="37">
         <f>STDEV(D11:I13)</f>
         <v>0.73208449814095855</v>
       </c>
-      <c r="M11" s="31">
+      <c r="M11" s="37">
         <f>QUARTILE(E11:J13,3)-QUARTILE(E11:J13,1)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="D12" s="17">
-        <v>4</v>
-      </c>
-      <c r="E12" s="17">
-        <v>5</v>
-      </c>
-      <c r="F12" s="17">
-        <v>4</v>
-      </c>
-      <c r="G12" s="17">
+    <row r="12" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A12" s="32"/>
+      <c r="B12" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="14">
+        <v>4</v>
+      </c>
+      <c r="E12" s="14">
+        <v>5</v>
+      </c>
+      <c r="F12" s="14">
+        <v>4</v>
+      </c>
+      <c r="G12" s="14">
         <v>3</v>
       </c>
-      <c r="H12" s="17">
-        <v>4</v>
-      </c>
-      <c r="I12" s="17">
+      <c r="H12" s="14">
+        <v>4</v>
+      </c>
+      <c r="I12" s="14">
         <v>3</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="16">
         <f t="shared" si="0"/>
         <v>3.8333333333333335</v>
       </c>
-      <c r="K12" s="32"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
+      <c r="K12" s="35"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
     </row>
-    <row r="13" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="22"/>
-      <c r="B13" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="D13" s="17">
-        <v>4</v>
-      </c>
-      <c r="E13" s="17">
-        <v>5</v>
-      </c>
-      <c r="F13" s="17">
-        <v>4</v>
-      </c>
-      <c r="G13" s="17">
+    <row r="13" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A13" s="33"/>
+      <c r="B13" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" s="14">
+        <v>4</v>
+      </c>
+      <c r="E13" s="14">
+        <v>5</v>
+      </c>
+      <c r="F13" s="14">
+        <v>4</v>
+      </c>
+      <c r="G13" s="14">
         <v>3</v>
       </c>
-      <c r="H13" s="17">
-        <v>4</v>
-      </c>
-      <c r="I13" s="17">
-        <v>5</v>
-      </c>
-      <c r="J13" s="19">
+      <c r="H13" s="14">
+        <v>4</v>
+      </c>
+      <c r="I13" s="14">
+        <v>5</v>
+      </c>
+      <c r="J13" s="16">
         <f t="shared" si="0"/>
         <v>4.166666666666667</v>
       </c>
-      <c r="K13" s="34"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
+      <c r="K13" s="36"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
     </row>
-    <row r="14" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="36" t="s">
+    <row r="14" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A14" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="B14" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="D14" s="24">
-        <v>5</v>
-      </c>
-      <c r="E14" s="24">
-        <v>5</v>
-      </c>
-      <c r="F14" s="24">
-        <v>5</v>
-      </c>
-      <c r="G14" s="24">
-        <v>5</v>
-      </c>
-      <c r="H14" s="24">
-        <v>4</v>
-      </c>
-      <c r="I14" s="24">
-        <v>4</v>
-      </c>
-      <c r="J14" s="26">
+      <c r="D14" s="19">
+        <v>5</v>
+      </c>
+      <c r="E14" s="19">
+        <v>5</v>
+      </c>
+      <c r="F14" s="19">
+        <v>5</v>
+      </c>
+      <c r="G14" s="19">
+        <v>5</v>
+      </c>
+      <c r="H14" s="19">
+        <v>4</v>
+      </c>
+      <c r="I14" s="19">
+        <v>4</v>
+      </c>
+      <c r="J14" s="21">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
-      <c r="K14" s="37">
+      <c r="K14" s="43">
         <f>AVERAGE(J14:J16)</f>
         <v>4.7777777777777777</v>
       </c>
-      <c r="L14" s="38">
+      <c r="L14" s="46">
         <f>STDEV(D14:I16)</f>
         <v>0.42779263194649864</v>
       </c>
-      <c r="M14" s="38">
+      <c r="M14" s="46">
         <f>QUARTILE(E14:J16,3)-QUARTILE(E14:J16,1)</f>
         <v>0.16666666666666696</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A15" s="39"/>
-      <c r="B15" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="D15" s="24">
-        <v>5</v>
-      </c>
-      <c r="E15" s="24">
-        <v>5</v>
-      </c>
-      <c r="F15" s="24">
-        <v>5</v>
-      </c>
-      <c r="G15" s="24">
-        <v>5</v>
-      </c>
-      <c r="H15" s="24">
-        <v>4</v>
-      </c>
-      <c r="I15" s="24">
-        <v>5</v>
-      </c>
-      <c r="J15" s="26">
+    <row r="15" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A15" s="41"/>
+      <c r="B15" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" s="19">
+        <v>5</v>
+      </c>
+      <c r="E15" s="19">
+        <v>5</v>
+      </c>
+      <c r="F15" s="19">
+        <v>5</v>
+      </c>
+      <c r="G15" s="19">
+        <v>5</v>
+      </c>
+      <c r="H15" s="19">
+        <v>4</v>
+      </c>
+      <c r="I15" s="19">
+        <v>5</v>
+      </c>
+      <c r="J15" s="21">
         <f t="shared" si="0"/>
         <v>4.833333333333333</v>
       </c>
-      <c r="K15" s="40"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="41"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="47"/>
     </row>
-    <row r="16" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="28" x14ac:dyDescent="0.15">
       <c r="A16" s="42"/>
-      <c r="B16" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="D16" s="24">
-        <v>4</v>
-      </c>
-      <c r="E16" s="24">
-        <v>5</v>
-      </c>
-      <c r="F16" s="24">
-        <v>5</v>
-      </c>
-      <c r="G16" s="24">
-        <v>5</v>
-      </c>
-      <c r="H16" s="24">
-        <v>5</v>
-      </c>
-      <c r="I16" s="24">
-        <v>5</v>
-      </c>
-      <c r="J16" s="26">
+      <c r="B16" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="D16" s="19">
+        <v>4</v>
+      </c>
+      <c r="E16" s="19">
+        <v>5</v>
+      </c>
+      <c r="F16" s="19">
+        <v>5</v>
+      </c>
+      <c r="G16" s="19">
+        <v>5</v>
+      </c>
+      <c r="H16" s="19">
+        <v>5</v>
+      </c>
+      <c r="I16" s="19">
+        <v>5</v>
+      </c>
+      <c r="J16" s="21">
         <f t="shared" si="0"/>
         <v>4.833333333333333</v>
       </c>
-      <c r="K16" s="43"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="44"/>
+      <c r="K16" s="45"/>
+      <c r="L16" s="48"/>
+      <c r="M16" s="48"/>
     </row>
-    <row r="17" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
+    <row r="17" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A17" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="B17" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="D17" s="17">
-        <v>4</v>
-      </c>
-      <c r="E17" s="17">
-        <v>5</v>
-      </c>
-      <c r="F17" s="17">
-        <v>5</v>
-      </c>
-      <c r="G17" s="17">
-        <v>4</v>
-      </c>
-      <c r="H17" s="17">
-        <v>5</v>
-      </c>
-      <c r="I17" s="17">
-        <v>5</v>
-      </c>
-      <c r="J17" s="19">
+      <c r="D17" s="14">
+        <v>4</v>
+      </c>
+      <c r="E17" s="14">
+        <v>5</v>
+      </c>
+      <c r="F17" s="14">
+        <v>5</v>
+      </c>
+      <c r="G17" s="14">
+        <v>4</v>
+      </c>
+      <c r="H17" s="14">
+        <v>5</v>
+      </c>
+      <c r="I17" s="14">
+        <v>5</v>
+      </c>
+      <c r="J17" s="16">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="34">
         <f>AVERAGE(J17:J23)</f>
         <v>4.4761904761904763</v>
       </c>
-      <c r="L17" s="31">
+      <c r="L17" s="37">
         <f>STDEV(D17:I23)</f>
         <v>0.74040513755103221</v>
       </c>
-      <c r="M17" s="31">
+      <c r="M17" s="37">
         <f>QUARTILE(E17:J23,3)-QUARTILE(E17:J23,1)</f>
         <v>0.66666666666666696</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="21"/>
-      <c r="B18" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="D18" s="17">
-        <v>4</v>
-      </c>
-      <c r="E18" s="17">
-        <v>5</v>
-      </c>
-      <c r="F18" s="17">
-        <v>4</v>
-      </c>
-      <c r="G18" s="17">
-        <v>5</v>
-      </c>
-      <c r="H18" s="17">
-        <v>5</v>
-      </c>
-      <c r="I18" s="17">
+    <row r="18" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A18" s="32"/>
+      <c r="B18" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D18" s="14">
+        <v>4</v>
+      </c>
+      <c r="E18" s="14">
+        <v>5</v>
+      </c>
+      <c r="F18" s="14">
+        <v>4</v>
+      </c>
+      <c r="G18" s="14">
+        <v>5</v>
+      </c>
+      <c r="H18" s="14">
+        <v>5</v>
+      </c>
+      <c r="I18" s="14">
         <v>3</v>
       </c>
-      <c r="J18" s="19">
+      <c r="J18" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K18" s="32"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="38"/>
     </row>
-    <row r="19" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A19" s="21"/>
-      <c r="B19" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="D19" s="17">
-        <v>4</v>
-      </c>
-      <c r="E19" s="17">
-        <v>5</v>
-      </c>
-      <c r="F19" s="17">
-        <v>5</v>
-      </c>
-      <c r="G19" s="17">
-        <v>5</v>
-      </c>
-      <c r="H19" s="17">
-        <v>4</v>
-      </c>
-      <c r="I19" s="17">
-        <v>5</v>
-      </c>
-      <c r="J19" s="19">
+    <row r="19" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A19" s="32"/>
+      <c r="B19" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D19" s="14">
+        <v>4</v>
+      </c>
+      <c r="E19" s="14">
+        <v>5</v>
+      </c>
+      <c r="F19" s="14">
+        <v>5</v>
+      </c>
+      <c r="G19" s="14">
+        <v>5</v>
+      </c>
+      <c r="H19" s="14">
+        <v>4</v>
+      </c>
+      <c r="I19" s="14">
+        <v>5</v>
+      </c>
+      <c r="J19" s="16">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
-      <c r="K19" s="32"/>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
+      <c r="K19" s="35"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="38"/>
     </row>
-    <row r="20" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A20" s="21"/>
-      <c r="B20" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="17">
-        <v>4</v>
-      </c>
-      <c r="E20" s="17">
-        <v>5</v>
-      </c>
-      <c r="F20" s="17">
-        <v>4</v>
-      </c>
-      <c r="G20" s="17">
-        <v>5</v>
-      </c>
-      <c r="H20" s="17">
-        <v>5</v>
-      </c>
-      <c r="I20" s="17">
+    <row r="20" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A20" s="32"/>
+      <c r="B20" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20" s="14">
+        <v>4</v>
+      </c>
+      <c r="E20" s="14">
+        <v>5</v>
+      </c>
+      <c r="F20" s="14">
+        <v>4</v>
+      </c>
+      <c r="G20" s="14">
+        <v>5</v>
+      </c>
+      <c r="H20" s="14">
+        <v>5</v>
+      </c>
+      <c r="I20" s="14">
         <v>3</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K20" s="32"/>
-      <c r="L20" s="33"/>
-      <c r="M20" s="33"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="38"/>
     </row>
-    <row r="21" spans="1:13" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="D21" s="17">
-        <v>4</v>
-      </c>
-      <c r="E21" s="17">
-        <v>5</v>
-      </c>
-      <c r="F21" s="17">
-        <v>5</v>
-      </c>
-      <c r="G21" s="17">
-        <v>4</v>
-      </c>
-      <c r="H21" s="17">
-        <v>5</v>
-      </c>
-      <c r="I21" s="17">
+    <row r="21" spans="1:13" ht="70" x14ac:dyDescent="0.15">
+      <c r="A21" s="32"/>
+      <c r="B21" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="D21" s="14">
+        <v>4</v>
+      </c>
+      <c r="E21" s="14">
+        <v>5</v>
+      </c>
+      <c r="F21" s="14">
+        <v>5</v>
+      </c>
+      <c r="G21" s="14">
+        <v>4</v>
+      </c>
+      <c r="H21" s="14">
+        <v>5</v>
+      </c>
+      <c r="I21" s="14">
         <v>3</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K21" s="32"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
+      <c r="K21" s="35"/>
+      <c r="L21" s="38"/>
+      <c r="M21" s="38"/>
     </row>
-    <row r="22" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="21"/>
-      <c r="B22" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="D22" s="17">
+    <row r="22" spans="1:13" ht="42" x14ac:dyDescent="0.15">
+      <c r="A22" s="32"/>
+      <c r="B22" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D22" s="14">
         <v>3</v>
       </c>
-      <c r="E22" s="17">
-        <v>5</v>
-      </c>
-      <c r="F22" s="17">
-        <v>5</v>
-      </c>
-      <c r="G22" s="17">
+      <c r="E22" s="14">
+        <v>5</v>
+      </c>
+      <c r="F22" s="14">
+        <v>5</v>
+      </c>
+      <c r="G22" s="14">
         <v>3</v>
       </c>
-      <c r="H22" s="17">
-        <v>5</v>
-      </c>
-      <c r="I22" s="17">
-        <v>5</v>
-      </c>
-      <c r="J22" s="19">
+      <c r="H22" s="14">
+        <v>5</v>
+      </c>
+      <c r="I22" s="14">
+        <v>5</v>
+      </c>
+      <c r="J22" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K22" s="32"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
+      <c r="K22" s="35"/>
+      <c r="L22" s="38"/>
+      <c r="M22" s="38"/>
     </row>
-    <row r="23" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="22"/>
-      <c r="B23" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="D23" s="17">
+    <row r="23" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A23" s="33"/>
+      <c r="B23" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D23" s="14">
         <v>3</v>
       </c>
-      <c r="E23" s="17">
-        <v>5</v>
-      </c>
-      <c r="F23" s="17">
-        <v>5</v>
-      </c>
-      <c r="G23" s="17">
-        <v>5</v>
-      </c>
-      <c r="H23" s="17">
-        <v>5</v>
-      </c>
-      <c r="I23" s="17">
-        <v>5</v>
-      </c>
-      <c r="J23" s="19">
+      <c r="E23" s="14">
+        <v>5</v>
+      </c>
+      <c r="F23" s="14">
+        <v>5</v>
+      </c>
+      <c r="G23" s="14">
+        <v>5</v>
+      </c>
+      <c r="H23" s="14">
+        <v>5</v>
+      </c>
+      <c r="I23" s="14">
+        <v>5</v>
+      </c>
+      <c r="J23" s="16">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
-      <c r="K23" s="34"/>
-      <c r="L23" s="35"/>
-      <c r="M23" s="35"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="39"/>
     </row>
-    <row r="24" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A24" s="45" t="s">
+    <row r="24" spans="1:13" ht="56" x14ac:dyDescent="0.15">
+      <c r="A24" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="C24" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="B24" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="D24" s="24">
-        <v>5</v>
-      </c>
-      <c r="E24" s="24">
+      <c r="D24" s="19">
+        <v>5</v>
+      </c>
+      <c r="E24" s="19">
         <v>3</v>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="19">
         <v>3</v>
       </c>
-      <c r="G24" s="24">
-        <v>5</v>
-      </c>
-      <c r="H24" s="24">
-        <v>4</v>
-      </c>
-      <c r="I24" s="24">
-        <v>4</v>
-      </c>
-      <c r="J24" s="26">
+      <c r="G24" s="19">
+        <v>5</v>
+      </c>
+      <c r="H24" s="19">
+        <v>4</v>
+      </c>
+      <c r="I24" s="19">
+        <v>4</v>
+      </c>
+      <c r="J24" s="21">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K24" s="29">
+      <c r="K24" s="22">
         <f>AVERAGE(D24:I24)</f>
         <v>4</v>
       </c>
-      <c r="L24" s="26">
+      <c r="L24" s="21">
         <f>STDEV(D24:I24)</f>
         <v>0.89442719099991586</v>
       </c>
-      <c r="M24" s="26">
+      <c r="M24" s="21">
         <f>QUARTILE(E24:J24,3)-QUARTILE(E24:J24,1)</f>
         <v>0.75</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="D25" s="17">
-        <v>4</v>
-      </c>
-      <c r="E25" s="17">
-        <v>5</v>
-      </c>
-      <c r="F25" s="17">
-        <v>4</v>
-      </c>
-      <c r="G25" s="17">
-        <v>5</v>
-      </c>
-      <c r="H25" s="17">
-        <v>5</v>
-      </c>
-      <c r="I25" s="17">
+    <row r="25" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A25" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D25" s="14">
+        <v>4</v>
+      </c>
+      <c r="E25" s="14">
+        <v>5</v>
+      </c>
+      <c r="F25" s="14">
+        <v>4</v>
+      </c>
+      <c r="G25" s="14">
+        <v>5</v>
+      </c>
+      <c r="H25" s="14">
+        <v>5</v>
+      </c>
+      <c r="I25" s="14">
         <v>3</v>
       </c>
-      <c r="J25" s="19">
+      <c r="J25" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K25" s="30">
+      <c r="K25" s="34">
         <f>AVERAGE(J25:J29)</f>
         <v>4.5333333333333332</v>
       </c>
-      <c r="L25" s="31">
+      <c r="L25" s="37">
         <f>STDEV(D25:I29)</f>
         <v>0.73029674334022221</v>
       </c>
-      <c r="M25" s="31">
+      <c r="M25" s="37">
         <f>QUARTILE(E25:J29,3)-QUARTILE(E25:J29,1)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A26" s="21"/>
-      <c r="B26" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="D26" s="17">
-        <v>4</v>
-      </c>
-      <c r="E26" s="17">
-        <v>5</v>
-      </c>
-      <c r="F26" s="17">
-        <v>4</v>
-      </c>
-      <c r="G26" s="17">
-        <v>4</v>
-      </c>
-      <c r="H26" s="17">
-        <v>5</v>
-      </c>
-      <c r="I26" s="17">
-        <v>4</v>
-      </c>
-      <c r="J26" s="19">
+    <row r="26" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A26" s="32"/>
+      <c r="B26" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="D26" s="14">
+        <v>4</v>
+      </c>
+      <c r="E26" s="14">
+        <v>5</v>
+      </c>
+      <c r="F26" s="14">
+        <v>4</v>
+      </c>
+      <c r="G26" s="14">
+        <v>4</v>
+      </c>
+      <c r="H26" s="14">
+        <v>5</v>
+      </c>
+      <c r="I26" s="14">
+        <v>4</v>
+      </c>
+      <c r="J26" s="16">
         <f t="shared" si="0"/>
         <v>4.333333333333333</v>
       </c>
-      <c r="K26" s="32"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
     </row>
-    <row r="27" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D27" s="17">
-        <v>5</v>
-      </c>
-      <c r="E27" s="17">
-        <v>5</v>
-      </c>
-      <c r="F27" s="17">
-        <v>5</v>
-      </c>
-      <c r="G27" s="17">
-        <v>5</v>
-      </c>
-      <c r="H27" s="17">
-        <v>5</v>
-      </c>
-      <c r="I27" s="17">
-        <v>4</v>
-      </c>
-      <c r="J27" s="19">
+    <row r="27" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A27" s="32"/>
+      <c r="B27" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="14">
+        <v>5</v>
+      </c>
+      <c r="E27" s="14">
+        <v>5</v>
+      </c>
+      <c r="F27" s="14">
+        <v>5</v>
+      </c>
+      <c r="G27" s="14">
+        <v>5</v>
+      </c>
+      <c r="H27" s="14">
+        <v>5</v>
+      </c>
+      <c r="I27" s="14">
+        <v>4</v>
+      </c>
+      <c r="J27" s="16">
         <f t="shared" si="0"/>
         <v>4.833333333333333</v>
       </c>
-      <c r="K27" s="32"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
+      <c r="K27" s="35"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="38"/>
     </row>
-    <row r="28" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A28" s="21"/>
-      <c r="B28" s="17" t="s">
+    <row r="28" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A28" s="32"/>
+      <c r="B28" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="D28" s="14">
+        <v>5</v>
+      </c>
+      <c r="E28" s="14">
+        <v>5</v>
+      </c>
+      <c r="F28" s="14">
+        <v>5</v>
+      </c>
+      <c r="G28" s="14">
+        <v>5</v>
+      </c>
+      <c r="H28" s="14">
+        <v>5</v>
+      </c>
+      <c r="I28" s="14">
+        <v>5</v>
+      </c>
+      <c r="J28" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K28" s="35"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="38"/>
+    </row>
+    <row r="29" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+      <c r="A29" s="33"/>
+      <c r="B29" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C29" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="D28" s="17">
-        <v>5</v>
-      </c>
-      <c r="E28" s="17">
-        <v>5</v>
-      </c>
-      <c r="F28" s="17">
-        <v>5</v>
-      </c>
-      <c r="G28" s="17">
-        <v>5</v>
-      </c>
-      <c r="H28" s="17">
-        <v>5</v>
-      </c>
-      <c r="I28" s="17">
-        <v>5</v>
-      </c>
-      <c r="J28" s="19">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="K28" s="32"/>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-    </row>
-    <row r="29" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="22"/>
-      <c r="B29" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="D29" s="17">
-        <v>5</v>
-      </c>
-      <c r="E29" s="17">
-        <v>5</v>
-      </c>
-      <c r="F29" s="17">
-        <v>5</v>
-      </c>
-      <c r="G29" s="17">
-        <v>4</v>
-      </c>
-      <c r="H29" s="17">
-        <v>4</v>
-      </c>
-      <c r="I29" s="17">
+      <c r="D29" s="14">
+        <v>5</v>
+      </c>
+      <c r="E29" s="14">
+        <v>5</v>
+      </c>
+      <c r="F29" s="14">
+        <v>5</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>4</v>
+      </c>
+      <c r="I29" s="14">
         <v>2</v>
       </c>
-      <c r="J29" s="19">
+      <c r="J29" s="16">
         <f t="shared" si="0"/>
         <v>4.166666666666667</v>
       </c>
-      <c r="K29" s="34"/>
-      <c r="L29" s="35"/>
-      <c r="M29" s="35"/>
+      <c r="K29" s="36"/>
+      <c r="L29" s="39"/>
+      <c r="M29" s="39"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="18">
+    <mergeCell ref="M11:M13"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="K11:K13"/>
+    <mergeCell ref="L11:L13"/>
     <mergeCell ref="A25:A29"/>
     <mergeCell ref="K25:K29"/>
     <mergeCell ref="L25:L29"/>
@@ -5167,12 +5177,6 @@
     <mergeCell ref="K17:K23"/>
     <mergeCell ref="L17:L23"/>
     <mergeCell ref="M17:M23"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="K11:K13"/>
-    <mergeCell ref="L11:L13"/>
-    <mergeCell ref="M11:M13"/>
   </mergeCells>
   <conditionalFormatting sqref="D8:I29">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
@@ -5185,48 +5189,48 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="28" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>114</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A2" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="11">
         <f>(0+2)/2</f>
         <v>1</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="11">
         <f>(3+5)/2</f>
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="11">
         <v>16</v>
       </c>
     </row>

</xml_diff>